<commit_message>
terminando depresion estructural decremental
</commit_message>
<xml_diff>
--- a/excel_de_info/NiMARE_Campos_Esenciales_v2.xlsx
+++ b/excel_de_info/NiMARE_Campos_Esenciales_v2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pablodeleon/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Applications/DataAnalysisNimare/excel_de_info/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F040343-1673-2F43-9E82-ED65287E983B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C54F063-9F8D-9C4E-A170-41C7B7231ED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GUIA_DE_CAMPOS" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="671" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="662" uniqueCount="192">
   <si>
     <t>GUÍA DE CAMPOS — META-ANÁLISIS NIMARE</t>
   </si>
@@ -879,10 +879,28 @@
     <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -895,28 +913,10 @@
     <xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1240,37 +1240,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
     </row>
     <row r="2" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
     </row>
     <row r="4" spans="1:7" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="12"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="12"/>
-      <c r="G4" s="12"/>
+      <c r="B4" s="16"/>
+      <c r="C4" s="16"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="16"/>
     </row>
     <row r="5" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
@@ -1503,15 +1503,15 @@
       </c>
     </row>
     <row r="16" spans="1:7" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="B16" s="12"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="12"/>
+      <c r="B16" s="16"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="16"/>
     </row>
     <row r="17" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
@@ -1703,42 +1703,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="22" t="s">
         <v>114</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
-      <c r="N1" s="12"/>
-      <c r="O1" s="12"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="16"/>
+      <c r="M1" s="16"/>
+      <c r="N1" s="16"/>
+      <c r="O1" s="16"/>
     </row>
     <row r="2" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
-      <c r="M2" s="12"/>
-      <c r="N2" s="12"/>
-      <c r="O2" s="12"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="16"/>
+      <c r="M2" s="16"/>
+      <c r="N2" s="16"/>
+      <c r="O2" s="16"/>
     </row>
     <row r="3" spans="1:15" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
@@ -1905,31 +1905,31 @@
       <c r="O6" s="9"/>
     </row>
     <row r="7" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="12" t="s">
         <v>151</v>
       </c>
-      <c r="B7" s="23">
+      <c r="B7" s="13">
         <v>-32</v>
       </c>
-      <c r="C7" s="23">
+      <c r="C7" s="13">
         <v>-70</v>
       </c>
-      <c r="D7" s="23">
+      <c r="D7" s="13">
         <v>56</v>
       </c>
-      <c r="E7" s="23">
+      <c r="E7" s="13">
         <v>168</v>
       </c>
-      <c r="F7" s="23" t="s">
-        <v>48</v>
-      </c>
-      <c r="G7" s="23" t="s">
+      <c r="F7" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="G7" s="13" t="s">
         <v>130</v>
       </c>
-      <c r="H7" s="23" t="s">
+      <c r="H7" s="13" t="s">
         <v>152</v>
       </c>
-      <c r="I7" s="23" t="s">
+      <c r="I7" s="13" t="s">
         <v>69</v>
       </c>
       <c r="J7" s="8"/>
@@ -1958,13 +1958,13 @@
       <c r="F8" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="G8" s="23" t="s">
+      <c r="G8" s="13" t="s">
         <v>130</v>
       </c>
       <c r="H8" s="7" t="s">
         <v>184</v>
       </c>
-      <c r="I8" s="23" t="s">
+      <c r="I8" s="13" t="s">
         <v>69</v>
       </c>
       <c r="J8" s="9"/>
@@ -1999,7 +1999,7 @@
       <c r="H9" s="7" t="s">
         <v>184</v>
       </c>
-      <c r="I9" s="23" t="s">
+      <c r="I9" s="13" t="s">
         <v>69</v>
       </c>
       <c r="J9" s="8"/>
@@ -2034,7 +2034,7 @@
       <c r="H10" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="I10" s="23" t="s">
+      <c r="I10" s="13" t="s">
         <v>69</v>
       </c>
       <c r="J10" s="9"/>
@@ -2045,31 +2045,17 @@
       <c r="O10" s="9"/>
     </row>
     <row r="11" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="7" t="s">
-        <v>183</v>
-      </c>
-      <c r="B11" s="7">
-        <v>-27.6</v>
-      </c>
-      <c r="C11" s="7">
-        <v>25.3</v>
-      </c>
-      <c r="D11" s="7">
-        <v>2.7</v>
-      </c>
-      <c r="E11" s="7">
-        <v>167</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="G11" s="7" t="s">
-        <v>129</v>
-      </c>
+      <c r="A11" s="7"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
       <c r="H11" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="I11" s="23" t="s">
+      <c r="I11" s="13" t="s">
         <v>69</v>
       </c>
       <c r="J11" s="8"/>
@@ -2104,7 +2090,7 @@
       <c r="H12" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="I12" s="23" t="s">
+      <c r="I12" s="13" t="s">
         <v>69</v>
       </c>
       <c r="J12" s="9"/>
@@ -2139,7 +2125,7 @@
       <c r="H13" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="I13" s="23" t="s">
+      <c r="I13" s="13" t="s">
         <v>69</v>
       </c>
       <c r="J13" s="8"/>
@@ -2174,7 +2160,7 @@
       <c r="H14" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="I14" s="23" t="s">
+      <c r="I14" s="13" t="s">
         <v>69</v>
       </c>
       <c r="J14" s="9"/>
@@ -2209,7 +2195,7 @@
       <c r="H15" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="I15" s="23" t="s">
+      <c r="I15" s="13" t="s">
         <v>69</v>
       </c>
       <c r="J15" s="8"/>
@@ -2244,7 +2230,7 @@
       <c r="H16" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="I16" s="23" t="s">
+      <c r="I16" s="13" t="s">
         <v>69</v>
       </c>
       <c r="J16" s="9"/>
@@ -2279,7 +2265,7 @@
       <c r="H17" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="I17" s="23" t="s">
+      <c r="I17" s="13" t="s">
         <v>69</v>
       </c>
       <c r="J17" s="8"/>
@@ -2314,7 +2300,7 @@
       <c r="H18" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="I18" s="23" t="s">
+      <c r="I18" s="13" t="s">
         <v>69</v>
       </c>
       <c r="J18" s="9"/>
@@ -2349,7 +2335,7 @@
       <c r="H19" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="I19" s="23" t="s">
+      <c r="I19" s="13" t="s">
         <v>69</v>
       </c>
       <c r="J19" s="8"/>
@@ -2360,31 +2346,17 @@
       <c r="O19" s="8"/>
     </row>
     <row r="20" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="7" t="s">
-        <v>186</v>
-      </c>
-      <c r="B20" s="7">
-        <v>-27.5</v>
-      </c>
-      <c r="C20" s="7">
-        <v>-6.5</v>
-      </c>
-      <c r="D20" s="7">
-        <v>2.5</v>
-      </c>
-      <c r="E20" s="7">
-        <v>93</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="G20" s="7" t="s">
-        <v>129</v>
-      </c>
+      <c r="A20" s="7"/>
+      <c r="B20" s="7"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="7"/>
       <c r="H20" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="I20" s="23" t="s">
+      <c r="I20" s="13" t="s">
         <v>69</v>
       </c>
       <c r="J20" s="9"/>
@@ -2395,31 +2367,17 @@
       <c r="O20" s="9"/>
     </row>
     <row r="21" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="7" t="s">
-        <v>186</v>
-      </c>
-      <c r="B21" s="7">
-        <v>27.5</v>
-      </c>
-      <c r="C21" s="7">
-        <v>-9.5</v>
-      </c>
-      <c r="D21" s="7">
-        <v>-4.5</v>
-      </c>
-      <c r="E21" s="7">
-        <v>93</v>
-      </c>
-      <c r="F21" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="G21" s="7" t="s">
-        <v>129</v>
-      </c>
+      <c r="A21" s="7"/>
+      <c r="B21" s="7"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="7"/>
       <c r="H21" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="I21" s="23" t="s">
+      <c r="I21" s="13" t="s">
         <v>69</v>
       </c>
       <c r="J21" s="8"/>
@@ -2933,42 +2891,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
-      <c r="N1" s="12"/>
-      <c r="O1" s="12"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="16"/>
+      <c r="M1" s="16"/>
+      <c r="N1" s="16"/>
+      <c r="O1" s="16"/>
     </row>
     <row r="2" spans="1:16" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
-      <c r="M2" s="12"/>
-      <c r="N2" s="12"/>
-      <c r="O2" s="12"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="16"/>
+      <c r="M2" s="16"/>
+      <c r="N2" s="16"/>
+      <c r="O2" s="16"/>
     </row>
     <row r="3" spans="1:16" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
@@ -5093,42 +5051,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="23" t="s">
         <v>131</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
-      <c r="N1" s="12"/>
-      <c r="O1" s="12"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="16"/>
+      <c r="M1" s="16"/>
+      <c r="N1" s="16"/>
+      <c r="O1" s="16"/>
     </row>
     <row r="2" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
-      <c r="M2" s="12"/>
-      <c r="N2" s="12"/>
-      <c r="O2" s="12"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="16"/>
+      <c r="M2" s="16"/>
+      <c r="N2" s="16"/>
+      <c r="O2" s="16"/>
     </row>
     <row r="3" spans="1:15" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
@@ -6016,42 +5974,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="24" t="s">
         <v>132</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
-      <c r="N1" s="12"/>
-      <c r="O1" s="12"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="16"/>
+      <c r="M1" s="16"/>
+      <c r="N1" s="16"/>
+      <c r="O1" s="16"/>
     </row>
     <row r="2" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
-      <c r="M2" s="12"/>
-      <c r="N2" s="12"/>
-      <c r="O2" s="12"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="16"/>
+      <c r="M2" s="16"/>
+      <c r="N2" s="16"/>
+      <c r="O2" s="16"/>
     </row>
     <row r="3" spans="1:15" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
@@ -6935,42 +6893,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="24" t="s">
         <v>133</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
-      <c r="N1" s="12"/>
-      <c r="O1" s="12"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="16"/>
+      <c r="M1" s="16"/>
+      <c r="N1" s="16"/>
+      <c r="O1" s="16"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" s="17" t="s">
         <v>136</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
-      <c r="M2" s="12"/>
-      <c r="N2" s="12"/>
-      <c r="O2" s="12"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="16"/>
+      <c r="M2" s="16"/>
+      <c r="N2" s="16"/>
+      <c r="O2" s="16"/>
     </row>
     <row r="3" spans="1:15" ht="26" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
@@ -6996,13 +6954,13 @@
       <c r="B4" s="7">
         <v>2</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C4" s="11" t="s">
         <v>138</v>
       </c>
-      <c r="D4" s="21" t="s">
+      <c r="D4" s="11" t="s">
         <v>147</v>
       </c>
-      <c r="E4" s="24" t="s">
+      <c r="E4" s="14" t="s">
         <v>157</v>
       </c>
     </row>
@@ -7019,7 +6977,7 @@
       <c r="D5" s="7" t="s">
         <v>150</v>
       </c>
-      <c r="E5" s="24" t="s">
+      <c r="E5" s="14" t="s">
         <v>157</v>
       </c>
     </row>
@@ -7036,7 +6994,7 @@
       <c r="D6" s="7" t="s">
         <v>155</v>
       </c>
-      <c r="E6" s="24" t="s">
+      <c r="E6" s="14" t="s">
         <v>157</v>
       </c>
     </row>
@@ -7047,13 +7005,13 @@
       <c r="B7" s="7">
         <v>7</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="C7" s="11" t="s">
         <v>159</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>160</v>
       </c>
-      <c r="E7" s="21" t="s">
+      <c r="E7" s="11" t="s">
         <v>161</v>
       </c>
     </row>
@@ -7064,13 +7022,13 @@
       <c r="B8" s="7">
         <v>9</v>
       </c>
-      <c r="C8" s="21" t="s">
+      <c r="C8" s="11" t="s">
         <v>167</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="E8" s="21" t="s">
+      <c r="E8" s="11" t="s">
         <v>165</v>
       </c>
     </row>
@@ -7087,7 +7045,7 @@
       <c r="D9" s="7" t="s">
         <v>172</v>
       </c>
-      <c r="E9" s="21" t="s">
+      <c r="E9" s="11" t="s">
         <v>169</v>
       </c>
     </row>
@@ -7115,13 +7073,13 @@
       <c r="B11" s="7">
         <v>13</v>
       </c>
-      <c r="C11" s="21" t="s">
+      <c r="C11" s="11" t="s">
         <v>179</v>
       </c>
       <c r="D11" s="7" t="s">
         <v>181</v>
       </c>
-      <c r="E11" s="21" t="s">
+      <c r="E11" s="11" t="s">
         <v>182</v>
       </c>
       <c r="F11" t="s">
@@ -7135,13 +7093,13 @@
       <c r="B12" s="7">
         <v>20</v>
       </c>
-      <c r="C12" s="21" t="s">
+      <c r="C12" s="11" t="s">
         <v>189</v>
       </c>
       <c r="D12" s="7" t="s">
         <v>190</v>
       </c>
-      <c r="E12" s="21" t="s">
+      <c r="E12" s="11" t="s">
         <v>191</v>
       </c>
     </row>

</xml_diff>